<commit_message>
Accurate peer-set percentiles for all stocks; promote & refresh Excel navigation tab
</commit_message>
<xml_diff>
--- a/Navrist_Feature_to_Dashboard_Map.xlsx
+++ b/Navrist_Feature_to_Dashboard_Map.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feature Map" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Section Overview" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Navigation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Navigation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feature Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Section Overview" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Map'!$A$2:$F$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Feature Map'!$A$2:$F$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,17 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +82,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D4ED8"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -127,6 +141,16 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -493,6 +517,427 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Navigation — where to tap to reach each feature   (Main tab → Sub-tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Looking for…</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Navigate (tap path)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Financial statements analysis</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Financial statements analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Revenue / profit trend analysis</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Revenue/profit trend analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Margin analysis</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Margin analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Quarterly results / KPI movement / PAT / Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Quarterly results analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Ratio analysis</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Ratio analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Valuation metrics (P/E, P/B, EV/EBITDA, P/E band)</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Valuation metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>ROE / ROCE analysis</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → ROE/ROCE analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Intrinsic / fair value / DCF / upside</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Intrinsic value / fair value estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Debt analysis / solvency score</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Debt &amp; Cash Flow → Debt analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Cash flow / FCF / CFO / Capex</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Debt &amp; Cash Flow → Cash flow analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Shareholding pattern</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Ownership → Shareholding pattern analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Promoter holding / pledge / governance risk</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Ownership → Promoter holding / pledge tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Institutional holding / FII / DII flows</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Ownership → Institutional holding / FII / DII tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Peer comparison (size &amp; sector-aware peers)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Market-cap class (Large / Mid / Small cap)</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison   (chip on each row; also next to the ticker in the header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>AI-suggested comparison parameters</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison   (“AI · What to compare &amp; why” box)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>See more peers (top 5 → all peers)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison   (“See N more peers” button)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Sector comparison / percentile standing</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Sector comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Business quality scoring</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>AI Insights → Business quality scoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Annual report / concall summary (monthly)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>AI Insights → Annual report / concall summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Earnings estimate / forecast</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>AI Insights → Earnings estimate / forecast support</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Red-flag / forensic accounting signals</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>AI Insights → Red-flag / forensic accounting signals</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Moat / quality assessment</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>AI Insights → Moat / quality assessment support</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Export / PDF research report</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Export → Export / report generation</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Anything — just search</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Search bar (top-right) → type the term → jumps you straight there</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -659,7 +1104,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Sector peer table with green/red best-worst markers per metric; TARGET row highlighted (blue) and Sector Median row highlighted (grey) with visible backgrounds.</t>
+          <t>Size &amp; sector-aware peer table from Screener.in: company-specific peers matched on industry AND market-cap (works for small/mid-caps, not just large index names). Columns: Market Cap, Price, P/E, ROCE, Qtr Profit &amp; Sales Growth (YoY), Div Yield. Each row tagged Large/Mid/Small cap; green/red best-worst markers; TARGET row highlighted + Peer Median row. Top 5 peers shown with a “See N more peers” toggle. An “AI · What to compare &amp; why” note names the sector and flags the parameters that matter most for this company type.</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1494,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Sector benchmark card with overall percentile + per-metric percentile bars + comparative tags.</t>
+          <t>Standing vs the stock’s real closest peers: overall percentile + per-metric percentile bars (ROCE, P/E, Profit Growth, Sales Growth) computed across the ACTUAL peer set — accurate for every stock (no more a meaningless 100th on every metric for non-index names) + comparative tags. Market-cap tier shown.</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1597,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1315,455 +1760,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Navigation — where to tap to reach each feature</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Looking for…</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Navigate (tap path)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Financial statements analysis</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth → Financial statements analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Ratio analysis</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation → Ratio analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Valuation metrics</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation → Valuation metrics</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Peer comparison</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Peer comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Revenue/profit trend analysis</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth → Revenue/profit trend analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Margin analysis</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth → Margin analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>ROE/ROCE analysis</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation → ROE/ROCE analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Debt analysis</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Debt &amp; Cash Flow → Debt analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Cash flow analysis</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Debt &amp; Cash Flow → Cash flow analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Shareholding pattern analysis</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Ownership → Shareholding pattern analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Promoter holding / pledge tracking</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Ownership → Promoter holding / pledge tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Institutional holding / FII / DII tracking</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Ownership → Institutional holding / FII / DII tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Quarterly results analysis</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth → Quarterly results analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Annual report / concall summary</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>AI Insights → Annual report / concall summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Earnings estimate / forecast support</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>AI Insights → Earnings estimate / forecast support</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Red-flag / forensic accounting signals</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>AI Insights → Red-flag / forensic accounting signals</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Sector comparison</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Sector comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Intrinsic value / fair value estimate</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation → Intrinsic value / fair value estimate</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Business quality scoring</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>AI Insights → Business quality scoring</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Moat / quality assessment support</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>AI Insights → Moat / quality assessment support</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>KPI movement / Quarter-end / PAT / Revenue</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth → Quarterly results analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Free Cash Flow (FCF) / CFO / Capex</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Debt &amp; Cash Flow → Cash flow analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>FII / DII flows</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Ownership → Institutional holding / FII / DII tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Promoter pledge / governance risk</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Ownership → Promoter holding / pledge tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Fair value / upside / DCF</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation → Intrinsic value / fair value estimate</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Monthly concall summaries</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>AI Insights → Annual report / concall summary (Concalls tabs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Or use the search bar (top-right) and type the term</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>→ jumps you straight there</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
WIP snapshot of antigravity uncommitted work
</commit_message>
<xml_diff>
--- a/Navrist_Feature_to_Dashboard_Map.xlsx
+++ b/Navrist_Feature_to_Dashboard_Map.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Navigation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="navigation" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Feature Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Section Overview" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Feature Map'!$A$2:$F$22</definedName>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +59,16 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -116,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -151,6 +160,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -517,410 +533,380 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Navigation — where to tap to reach each feature   (Main tab → Sub-tab)</t>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Quick Navigation — Find Any Feature</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Looking for…</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>Navigate (tap path)</t>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Tap path (Main Tab → Sub-tab)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="n">
+      <c r="A3" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Financial statements analysis</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Financial statements (5Y/12Q)</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth → Financial statements analysis</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Revenue / profit trend analysis</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Revenue &amp; PAT growth / CAGR</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth → Revenue/profit trend analysis</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Margin analysis</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Gross / EBITDA / Operating margin</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth → Margin analysis</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Quarterly results / KPI movement / PAT / Revenue</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Quarterly results / KPI / Beat/Miss</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth → Quarterly results analysis</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Ratio analysis</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>ROE / ROCE ratios</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation → Ratio analysis</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Valuation metrics (P/E, P/B, EV/EBITDA, P/E band)</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>P/E, P/B, EV/EBITDA, FCF yield</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation → Valuation metrics</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>ROE / ROCE analysis</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Return-ratio chart (ROE/ROCE)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation → ROE/ROCE analysis</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>Intrinsic / fair value / DCF / upside</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Fair value / DCF / Upside</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation → Intrinsic value / fair value estimate</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Debt analysis / solvency score</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Debt / D:E / Solvency score</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Debt &amp; Cash Flow → Debt analysis</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Cash flow / FCF / CFO / Capex</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Debt &amp; Cash Flow → Cash flow analysis</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Shareholding pattern</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Ownership split / 12Q trend</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Ownership → Shareholding pattern analysis</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>Promoter holding / pledge / governance risk</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Promoter holding / Pledge %</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Ownership → Promoter holding / pledge tracking</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Institutional holding / FII / DII flows</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>FII / DII flows &amp; trends</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Ownership → Institutional holding / FII / DII tracking</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Peer comparison (size &amp; sector-aware peers)</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Peer comparison (size/sector)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Peers &amp; Sector → Peer comparison</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Market-cap class (Large / Mid / Small cap)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Peer comparison   (chip on each row; also next to the ticker in the header)</t>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Market-cap class (Large/Mid/Small)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>AI-suggested comparison parameters</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Peer comparison   (“AI · What to compare &amp; why” box)</t>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Percentile vs peers</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Sector comparison</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>See more peers (top 5 → all peers)</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Peer comparison   (“See N more peers” button)</t>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Concall transcripts (monthly)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Annual report / concall summary</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Sector comparison / percentile standing</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector → Sector comparison</t>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Quality score (0-100)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Business quality scoring</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Business quality scoring</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>AI Insights → Business quality scoring</t>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Moat / Pricing power</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Moat / quality assessment support</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Annual report / concall summary (monthly)</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>AI Insights → Annual report / concall summary</t>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Red flags / Forensic checks</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Red-flag / forensic accounting signals</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="15" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Earnings estimate / forecast</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>5-year forecast / Bull-Base-Bear</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>AI Insights → Earnings estimate / forecast support</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n">
+      <c r="A24" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Red-flag / forensic accounting signals</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>AI Insights → Red-flag / forensic accounting signals</t>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>PDF report / Export</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Export → Export / report generation</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="A25" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>Moat / quality assessment</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>AI Insights → Moat / quality assessment support</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="11" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>Export / PDF research report</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>Export → Export / report generation</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>Anything — just search</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>Search bar (top-right) → type the term → jumps you straight there</t>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Search anything</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Search bar (top-right) → type term → jumps to it</t>
         </is>
       </c>
     </row>
@@ -941,650 +927,570 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Navrist Research Terminal — Fundamental Research: Feature → Dashboard Map</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard Section (Tab)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Sub-tab (click inside the section)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Main Tab</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>Result shown (expected)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>Delivered in dashboard</t>
         </is>
       </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Navigate (tap path)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Financial statements analysis</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Financial statements analysis</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Clean statements tab, 5Y/12Q trend charts, key movement summary</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Income/Balance/Cash-flow tables with Annual (5Y) &amp; Quarterly (12Q) toggle + Revenue &amp; Net Profit trend chart + Key-Movement summary card (Revenue/PAT YoY).</t>
+      <c r="E3" s="12" t="inlineStr"/>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Financial statements analysis</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Ratio analysis</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Ratio analysis</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Ratio dashboard, trend lines, peer percentile view</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Ratio dashboard cards (ROE, ROCE, Operating Margin, D/E, Revenue Growth) + ROE/ROCE return-ratio trend chart + embedded Peer Percentile View (also shown here, not only in Peers &amp; Sector).</t>
+      <c r="E4" s="12" t="inlineStr"/>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Ratio analysis</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Valuation metrics</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Valuation metrics</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Valuation card, historical band chart, peer valuation table</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Valuation cards (P/E, P/B, P/S, EV/EBITDA, FCF yield) + Historical P/E Band chart (5Y, derived free from price history / INR EPS, with tappable 5Y Low/Median/High/Current levels + hover read-out) + peer valuation (P/E) table vs sector median.</t>
+      <c r="E5" s="12" t="inlineStr"/>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Valuation metrics</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Peer comparison</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>Peers &amp; Sector</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Peer comparison</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Peer table, best/worst markers, ranking strip</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Size &amp; sector-aware peer table from Screener.in: company-specific peers matched on industry AND market-cap (works for small/mid-caps, not just large index names). Columns: Market Cap, Price, P/E, ROCE, Qtr Profit &amp; Sales Growth (YoY), Div Yield. Each row tagged Large/Mid/Small cap; green/red best-worst markers; TARGET row highlighted + Peer Median row. Top 5 peers shown with a “See N more peers” toggle. An “AI · What to compare &amp; why” note names the sector and flags the parameters that matter most for this company type.</t>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Peer table, best/worst markers, size/sector-aware peers</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Peer comparison</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Revenue/profit trend analysis</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Revenue/profit trend analysis</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Growth trend charts, acceleration tags</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>YoY/QoQ revenue growth trend chart + quarterly table + growth-velocity tag + CAGR (3Y Revenue/PAT) &amp; growth-acceleration cards. YoY/QoQ shown with consistent ▲/▼ colour format.</t>
+      <c r="E7" s="12" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Revenue/profit trend analysis</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Margin analysis</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Margin analysis</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Margin panel, margin bridge, improving/stable/deteriorating tag</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Margin panel: 4-line Gross/EBITDA/EBIT/PAT trend chart + annual table + IMPROVING/STABLE/DETERIORATING tag. (Margin bridge optional/pending.)</t>
+      <c r="E8" s="12" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Margin analysis</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>ROE/ROCE analysis</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>ROE/ROCE analysis</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Return-ratio chart, quality commentary, peer context</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Return-ratio chart (ROE/ROCE) + ROE/ROCE table ABOVE the AI quality commentary (Groq). Peer context also in Peers &amp; Sector.</t>
+      <c r="E9" s="12" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → ROE/ROCE analysis</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Debt analysis</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Debt &amp; Cash Flow</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Debt analysis</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Debt panel, solvency score, risk alerts</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Debt Panel (D/E, Net Debt/EBITDA, Interest Coverage, Total Debt, Cash) + 0-100 Solvency Score (STRONG/MODERATE/WEAK) + separate Risk Alerts card.</t>
+      <c r="E10" s="12" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Debt &amp; Cash Flow → Debt analysis</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Cash flow analysis</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Debt &amp; Cash Flow</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Cash flow analysis</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Cash-conversion chart, FCF trend, warning flags</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Four cards (CFO/PAT, Operating CFO, Capex, Free Cash Flow) + Operating CF &amp; FCF trend chart + cash-flow warning-flags card.</t>
+      <c r="E11" s="12" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Debt &amp; Cash Flow → Cash flow analysis</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Shareholding pattern analysis</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Ownership</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Shareholding pattern analysis</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Ownership trend chart, change summary</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Ownership split (promoter / FII / DII / public) + composition bar + REAL 12-quarter Ownership Trend chart + QoQ change summary. Live from Screener.in.</t>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Ownership → Shareholding pattern analysis</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Promoter holding / pledge tracking</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Ownership</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Promoter holding / pledge tracking</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Promoter trend card, pledge alert, risk marker</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Promoter stake / pledged % / shares-pledged cards + pledge colour index (green/amber/red) + Governance Risk Marker card (LOW/MODERATE/HIGH) + REAL 12-quarter promoter-holding trend (Screener). Pledge from NSE (0% when none on record).</t>
+      <c r="E13" s="12" t="inlineStr"/>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Ownership → Promoter holding / pledge tracking</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Institutional holding / FII / DII tracking</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Ownership</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Institutional holding / FII / DII tracking</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Institutional flow trend, increasing/reducing interest tag</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>FII &amp; DII daily net-flow cards (live NSE session) + interest tags + REAL 12-quarter FII/DII holding-trend chart with increasing/reducing tags (Screener) + stock institutional ownership %.</t>
+      <c r="E14" s="12" t="inlineStr"/>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Ownership → Institutional holding / FII / DII tracking</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Quarterly results analysis</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Statements &amp; Growth</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Quarterly results analysis</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Result snapshot, beat/miss summary, KPI movement table</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Result Snapshot card (Revenue/PAT/Operating Margin) + Beat/Miss summary (PEAD) + KPI Movement table (Revenue/PAT/Margin QoQ &amp; YoY) + Recent Quarters detail.</t>
+      <c r="E15" s="12" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Statements &amp; Growth → Quarterly results analysis</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Annual report / concall summary</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>AI Insights</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Annual report / concall summary</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Structured summary with key sections</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>PER-MONTH 'Concalls' tabs (like Screener): each month's earnings call grounded in its REAL transcript (Screener -&gt; BSE PDF, pypdf) summarised by Groq into summary, financial highlights, growth drivers, business wins, risks, guidance &amp; management tone. Latest is pre-computed; older months summarise on click.</t>
+      <c r="E16" s="12" t="inlineStr"/>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Annual report / concall summary</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Earnings estimate / forecast support</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>AI Insights</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Earnings estimate / forecast support</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Internal forecast table, scenario view, confidence note</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Interactive 5Y forecast table + Bull/Base/Bear scenario selector + growth slider + confidence note.</t>
+      <c r="E17" s="12" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Earnings estimate / forecast support</t>
         </is>
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Red-flag / forensic accounting signals</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>AI Insights</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Red-flag / forensic accounting signals</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Red-flag checklist with severity score</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Forensic checklist (CFO vs PAT, dilution, receivables, asset quality) with PASS/WARN/FAIL + severity index + overall risk level.</t>
+      <c r="E18" s="12" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Red-flag / forensic accounting signals</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Sector comparison</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Peers &amp; Sector</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Sector comparison</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Sector benchmark card, percentile view</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Standing vs the stock’s real closest peers: overall percentile + per-metric percentile bars (ROCE, P/E, Profit Growth, Sales Growth) computed across the ACTUAL peer set — accurate for every stock (no more a meaningless 100th on every metric for non-index names) + comparative tags. Market-cap tier shown.</t>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Sector benchmark card, percentile view (accurate for all stocks)</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Peers &amp; Sector → Sector comparison</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Intrinsic value / fair value estimate</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>Ratios &amp; Valuation</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Intrinsic value / fair value estimate</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>Fair-value range, upside/downside, sensitivity table</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Fair-value range (Bear-Bull) + Base fair value + current price + Upside/Downside vs price + reverse-DCF sensitivity matrix.</t>
+      <c r="E20" s="12" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Ratios &amp; Valuation → Intrinsic value / fair value estimate</t>
         </is>
       </c>
     </row>
     <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Business quality scoring</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>AI Insights</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Business quality scoring</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>0-100 quality score, sub-scores, rationale chips</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>0-100 quality score gauge (gradient ring) + rationale chips + quality sub-scores (Profitability, Balance-sheet, Cash conversion, Growth).</t>
+      <c r="E21" s="12" t="inlineStr"/>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Business quality scoring</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Moat / quality assessment support</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>AI Insights</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Moat / quality assessment support</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Structured moat memo, confidence level</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Moat audit: classification + confidence-level gauge (with %) + pricing-power &amp; barriers-to-entry meters + structured moat memo.</t>
+      <c r="E22" s="12" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>AI Insights → Moat / quality assessment support</t>
         </is>
       </c>
     </row>
@@ -1595,169 +1501,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Dashboard Sections (top tabs) and their feature sub-tabs</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Section (top tab)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Feature sub-tabs (in order)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="72" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Statements &amp; Growth</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Financial statements analysis
-  •  Revenue/profit trend analysis
-  •  Margin analysis
-  •  Quarterly results analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="72" customHeight="1">
-      <c r="A4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Ratios &amp; Valuation</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Ratio analysis
-  •  Valuation metrics
-  •  ROE/ROCE analysis
-  •  Intrinsic value / fair value estimate</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Debt &amp; Cash Flow</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Debt analysis
-  •  Cash flow analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Ownership</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Shareholding pattern analysis
-  •  Promoter holding / pledge tracking
-  •  Institutional holding / FII / DII tracking</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Peers &amp; Sector</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Peer comparison
-  •  Sector comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="88" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>AI Insights</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Annual report / concall summary
-  •  Earnings estimate / forecast support
-  •  Red-flag / forensic accounting signals
-  •  Business quality scoring
-  •  Moat / quality assessment support</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  •  Export / report generation (PDF research report)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>